<commit_message>
Plan: GitHub access and push done
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JZeYZyS68Qg1mcBtJkp6XV
</commit_message>
<xml_diff>
--- a/docs/VerifiCasa-plan.xlsx
+++ b/docs/VerifiCasa-plan.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="187">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="187">
   <si>
     <t xml:space="preserve">VerifiCasa — work plan</t>
   </si>
@@ -156,33 +156,36 @@
     <t xml:space="preserve">P0 – now</t>
   </si>
   <si>
+    <t xml:space="preserve">Sign in as iamvava7 → github.com/apps/claude/installations/select_target → iamvava7 → repo 'yes'. If still blocked, start a new session with iamvava7/yes selected.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Push the 3 waiting SpaceTwin commits (tour page, tour quality, Maria)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Claude</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Branch 'spacetwin'. Backup: spacetwin-unpushed.bundle (git pull &lt;bundle&gt; spacetwin).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Make repos private (if still wanted)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P2 – later</t>
+  </si>
+  <si>
     <t xml:space="preserve">To do</t>
   </si>
   <si>
-    <t xml:space="preserve">Sign in as iamvava7 → github.com/apps/claude/installations/select_target → iamvava7 → repo 'yes'. If still blocked, start a new session with iamvava7/yes selected.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Push the 3 waiting SpaceTwin commits (tour page, tour quality, Maria)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Claude</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Branch 'spacetwin'. Backup: spacetwin-unpushed.bundle (git pull &lt;bundle&gt; spacetwin).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Make repos private (if still wanted)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P2 – later</t>
-  </si>
-  <si>
     <t xml:space="preserve">GitHub → repo → Settings → Danger zone → Change visibility. Testers then need an invite to clone.</t>
   </si>
   <si>
@@ -364,9 +367,6 @@
   </si>
   <si>
     <t xml:space="preserve">Tour page rebuilt from Figma 'Web · 3D Tour viewer' (PC + phone, details panel, room strip, loading)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No – waiting T02</t>
   </si>
   <si>
     <t xml:space="preserve">6701ee7</t>
@@ -731,12 +731,16 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -764,7 +768,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -781,11 +785,19 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="12">
+  <dxfs count="13">
     <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FF0E7C5A"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFDFF3EA"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -801,6 +813,14 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FF000000"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF6B7280"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -856,14 +876,6 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FF0000FF"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFDFF3EA"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -1133,178 +1145,178 @@
   <dimension ref="A1:B25"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="46"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="4" t="n">
+      <c r="B5" s="5" t="n">
         <f aca="false">COUNTA(Tasks!A2:A58)</f>
         <v>17</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="4" t="n">
+      <c r="B6" s="5" t="n">
         <f aca="false">COUNTIF(Tasks!F2:F58,"Done")</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="4" t="n">
+      <c r="B7" s="5" t="n">
         <f aca="false">COUNTIF(Tasks!F2:F58,"Blocked")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="4" t="n">
+      <c r="B8" s="5" t="n">
         <f aca="false">COUNTIFS(Tasks!D2:D58,"You",Tasks!F2:F58,"&lt;&gt;Done")</f>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" s="5" t="n">
+        <f aca="false">COUNTIFS(Tasks!D2:D58,"Claude",Tasks!F2:F58,"&lt;&gt;Done")</f>
         <v>7</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B9" s="4" t="n">
-        <f aca="false">COUNTIFS(Tasks!D2:D58,"Claude",Tasks!F2:F58,"&lt;&gt;Done")</f>
-        <v>8</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="4" t="n">
+      <c r="B10" s="5" t="n">
         <f aca="false">COUNTIFS(Tasks!E2:E58,"P0 – now",Tasks!F2:F58,"&lt;&gt;Done")</f>
-        <v>4</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B11" s="5" t="n">
+      <c r="B11" s="6" t="n">
         <f aca="false">IF(B5=0,0,B6/B5)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4"/>
-      <c r="B12" s="4"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="s">
+        <v>0.117647058823529</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="5"/>
+      <c r="B12" s="5"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="3"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4" t="s">
+      <c r="B13" s="4"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="4"/>
-    </row>
-    <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="s">
+      <c r="B14" s="5"/>
+    </row>
+    <row r="15" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="4"/>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4" t="s">
+      <c r="B15" s="5"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B16" s="4"/>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="s">
+      <c r="B16" s="5"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B17" s="4"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4" t="s">
+      <c r="B17" s="5"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B18" s="4"/>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4"/>
-      <c r="B19" s="4"/>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="3" t="s">
+      <c r="B18" s="5"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="5"/>
+      <c r="B19" s="5"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B20" s="3"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4" t="s">
+      <c r="B20" s="4"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B21" s="4" t="s">
+      <c r="B21" s="5" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="4" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="B22" s="5" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="4" t="s">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B23" s="4" t="s">
+      <c r="B23" s="5" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="4" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="B24" s="4" t="s">
+      <c r="B24" s="5" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="4" t="s">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="B25" s="4" t="s">
+      <c r="B25" s="5" t="s">
         <v>27</v>
       </c>
     </row>
@@ -1327,506 +1339,510 @@
   <dimension ref="A1:I18"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="5" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="60"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="5" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="12"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="6" t="s">
+    <row r="1" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="F1" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="G1" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="H1" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="I1" s="7" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="4" t="s">
+    <row r="2" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="G2" s="5"/>
+      <c r="H2" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4" t="s">
+      <c r="I2" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="I2" s="4"/>
-    </row>
-    <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4" t="s">
+    </row>
+    <row r="3" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="F3" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="G3" s="4" t="s">
+      <c r="F3" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="G3" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="H3" s="4" t="s">
+      <c r="H3" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="I3" s="4"/>
-    </row>
-    <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
+      <c r="I3" s="5" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="F4" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="G4" s="4" t="s">
+      <c r="F4" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="G4" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="H4" s="4" t="s">
+      <c r="H4" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I4" s="5"/>
+    </row>
+    <row r="5" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="F5" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="I4" s="4"/>
-    </row>
-    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="B5" s="4" t="s">
+      <c r="G5" s="5"/>
+      <c r="H5" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="I5" s="5"/>
+    </row>
+    <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="G6" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="H6" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="I6" s="5"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="B7" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="C7" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="I7" s="5"/>
+    </row>
+    <row r="8" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="D8" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="E5" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="G5" s="4"/>
-      <c r="H5" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="I5" s="4"/>
-    </row>
-    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="G6" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="H6" s="4" t="s">
+      <c r="E8" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="I8" s="5"/>
+    </row>
+    <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="G9" s="5"/>
+      <c r="H9" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="I9" s="5"/>
+    </row>
+    <row r="10" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="H10" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="I10" s="5"/>
+    </row>
+    <row r="11" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="G11" s="5"/>
+      <c r="H11" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="I11" s="5"/>
+    </row>
+    <row r="12" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="D12" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="I6" s="4"/>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="C7" s="4" t="s">
+      <c r="E12" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="G12" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="H12" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="I12" s="5"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="G13" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="H13" s="5"/>
+      <c r="I13" s="5"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="D14" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="E7" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="G7" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="H7" s="4" t="s">
+      <c r="E14" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="F14" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="G14" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="H14" s="5"/>
+      <c r="I14" s="5"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="F15" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="G15" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="H15" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="I15" s="5"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="F16" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="G16" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="H16" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="I16" s="5"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="E17" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="I7" s="4"/>
-    </row>
-    <row r="8" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="D8" s="4" t="s">
+      <c r="F17" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="G17" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="H17" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="I17" s="5"/>
+    </row>
+    <row r="18" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="D18" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="E8" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="G8" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="H8" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="I8" s="4"/>
-    </row>
-    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="G9" s="4"/>
-      <c r="H9" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="I9" s="4"/>
-    </row>
-    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="C10" s="4" t="s">
+      <c r="E18" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="F18" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="G18" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="D10" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="F10" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="G10" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="H10" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="I10" s="4"/>
-    </row>
-    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="E11" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="F11" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="G11" s="4"/>
-      <c r="H11" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="I11" s="4"/>
-    </row>
-    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="F12" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="G12" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="H12" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="I12" s="4"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="E13" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="F13" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="G13" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="H13" s="4"/>
-      <c r="I13" s="4"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="E14" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="F14" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="G14" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="H14" s="4"/>
-      <c r="I14" s="4"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="D15" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="E15" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="F15" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="G15" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="H15" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="I15" s="4"/>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="D16" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="E16" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="F16" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="G16" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="H16" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="I16" s="4"/>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="B17" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="D17" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="E17" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="F17" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="G17" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="H17" s="4" t="s">
-        <v>95</v>
-      </c>
-      <c r="I17" s="4"/>
-    </row>
-    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="B18" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="D18" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="E18" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="F18" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="G18" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="H18" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="I18" s="4"/>
+      <c r="H18" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="I18" s="5"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:I18"/>
   <conditionalFormatting sqref="A2:I58">
-    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="5">
+    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>$F2="Done"</formula>
     </cfRule>
-    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
+    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>$F2="Blocked"</formula>
     </cfRule>
-    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
+    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
       <formula>$F2="In progress"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D2:D58">
-    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
       <formula>$D2="You"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1863,129 +1879,129 @@
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="90"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="90"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="18"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="B1" s="6" t="s">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="B1" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="C1" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="D1" s="7" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="4" t="s">
+      <c r="E1" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="B2" s="4" t="s">
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="B2" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="C2" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="D2" s="5" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="B3" s="4" t="s">
+      <c r="E2" s="5" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="B3" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="E3" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="D3" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="B4" s="4" t="s">
+    </row>
+    <row r="4" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="B4" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="C4" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="E4" s="4" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="B5" s="4" t="s">
+      <c r="E4" s="5" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="B5" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="C5" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="E5" s="4" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
+      <c r="E5" s="5" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="E6" s="5" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="5" t="s">
         <v>122</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="E7" s="5" t="s">
         <v>125</v>
       </c>
     </row>
@@ -2008,425 +2024,425 @@
   <dimension ref="A1:H18"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="55"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="16"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="6" t="s">
+    <row r="1" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="7" t="s">
         <v>126</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="7" t="s">
         <v>127</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="7" t="s">
         <v>128</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="7" t="s">
         <v>129</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="F1" s="7" t="s">
         <v>131</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="G1" s="7" t="s">
         <v>132</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="H1" s="7" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="4" t="n">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="5" t="s">
         <v>134</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="5" t="s">
         <v>136</v>
       </c>
-      <c r="E2" s="7" t="n">
+      <c r="E2" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="F2" s="7" t="n">
+      <c r="F2" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G2" s="4" t="n">
+      <c r="G2" s="5" t="n">
         <f aca="false">E2*2-F2</f>
         <v>8</v>
       </c>
-      <c r="H2" s="4"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4" t="n">
+      <c r="H2" s="5"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="5" t="s">
         <v>137</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="5" t="s">
         <v>138</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="5" t="s">
         <v>139</v>
       </c>
-      <c r="E3" s="7" t="n">
+      <c r="E3" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="F3" s="7" t="n">
+      <c r="F3" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G3" s="4" t="n">
+      <c r="G3" s="5" t="n">
         <f aca="false">E3*2-F3</f>
         <v>8</v>
       </c>
-      <c r="H3" s="4"/>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="n">
+      <c r="H3" s="5"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="5" t="s">
         <v>141</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="5" t="s">
         <v>142</v>
       </c>
-      <c r="E4" s="7" t="n">
+      <c r="E4" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="F4" s="7" t="n">
+      <c r="F4" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="G4" s="4" t="n">
+      <c r="G4" s="5" t="n">
         <f aca="false">E4*2-F4</f>
         <v>7</v>
       </c>
-      <c r="H4" s="4"/>
-    </row>
-    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="n">
+      <c r="H4" s="5"/>
+    </row>
+    <row r="5" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="E5" s="7" t="n">
+      <c r="E5" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="F5" s="7" t="n">
+      <c r="F5" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G5" s="4" t="n">
+      <c r="G5" s="5" t="n">
         <f aca="false">E5*2-F5</f>
         <v>8</v>
       </c>
-      <c r="H5" s="4"/>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="n">
+      <c r="H5" s="5"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="5" t="s">
         <v>147</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="5" t="s">
         <v>148</v>
       </c>
-      <c r="E6" s="7" t="n">
+      <c r="E6" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="F6" s="7" t="n">
+      <c r="F6" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G6" s="4" t="n">
+      <c r="G6" s="5" t="n">
         <f aca="false">E6*2-F6</f>
         <v>6</v>
       </c>
-      <c r="H6" s="4"/>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="n">
+      <c r="H6" s="5"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="5" t="s">
         <v>149</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="E7" s="7" t="n">
+      <c r="E7" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="F7" s="7" t="n">
+      <c r="F7" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="G7" s="4" t="n">
+      <c r="G7" s="5" t="n">
         <f aca="false">E7*2-F7</f>
         <v>5</v>
       </c>
-      <c r="H7" s="4"/>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="n">
+      <c r="H7" s="5"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="D8" s="5" t="s">
         <v>154</v>
       </c>
-      <c r="E8" s="7" t="n">
+      <c r="E8" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="F8" s="7" t="n">
+      <c r="F8" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="G8" s="4" t="n">
+      <c r="G8" s="5" t="n">
         <f aca="false">E8*2-F8</f>
         <v>5</v>
       </c>
-      <c r="H8" s="4"/>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="n">
+      <c r="H8" s="5"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="5" t="s">
         <v>155</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="5" t="s">
         <v>156</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="D9" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="E9" s="7" t="n">
+      <c r="E9" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="F9" s="7" t="n">
+      <c r="F9" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G9" s="4" t="n">
+      <c r="G9" s="5" t="n">
         <f aca="false">E9*2-F9</f>
         <v>6</v>
       </c>
-      <c r="H9" s="4"/>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="n">
+      <c r="H9" s="5"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="5" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="D10" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="E10" s="7" t="n">
+      <c r="E10" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="F10" s="7" t="n">
+      <c r="F10" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G10" s="4" t="n">
+      <c r="G10" s="5" t="n">
         <f aca="false">E10*2-F10</f>
         <v>4</v>
       </c>
-      <c r="H10" s="4"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="n">
+      <c r="H10" s="5"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="5" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="5" t="s">
         <v>162</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="D11" s="5" t="s">
         <v>163</v>
       </c>
-      <c r="E11" s="7" t="n">
+      <c r="E11" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="F11" s="7" t="n">
+      <c r="F11" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="G11" s="4" t="n">
+      <c r="G11" s="5" t="n">
         <f aca="false">E11*2-F11</f>
         <v>2</v>
       </c>
-      <c r="H11" s="4"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="n">
+      <c r="H11" s="5"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="5" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="5" t="s">
         <v>164</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="C12" s="5" t="s">
         <v>165</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="D12" s="5" t="s">
         <v>166</v>
       </c>
-      <c r="E12" s="7" t="n">
+      <c r="E12" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="F12" s="7" t="n">
+      <c r="F12" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G12" s="4" t="n">
+      <c r="G12" s="5" t="n">
         <f aca="false">E12*2-F12</f>
         <v>6</v>
       </c>
-      <c r="H12" s="4"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="n">
+      <c r="H12" s="5"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="5" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="5" t="s">
         <v>167</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="5" t="s">
         <v>168</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="D13" s="5" t="s">
         <v>169</v>
       </c>
-      <c r="E13" s="7" t="n">
+      <c r="E13" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="F13" s="7" t="n">
+      <c r="F13" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G13" s="4" t="n">
+      <c r="G13" s="5" t="n">
         <f aca="false">E13*2-F13</f>
         <v>4</v>
       </c>
-      <c r="H13" s="4"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4" t="n">
+      <c r="H13" s="5"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="5" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="C14" s="5" t="s">
         <v>171</v>
       </c>
-      <c r="D14" s="4" t="s">
+      <c r="D14" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="E14" s="7" t="n">
+      <c r="E14" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="F14" s="7" t="n">
+      <c r="F14" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="G14" s="4" t="n">
+      <c r="G14" s="5" t="n">
         <f aca="false">E14*2-F14</f>
         <v>3</v>
       </c>
-      <c r="H14" s="4"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="n">
+      <c r="H14" s="5"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="5" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="5" t="s">
         <v>172</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="C15" s="5" t="s">
         <v>173</v>
       </c>
-      <c r="D15" s="4" t="s">
+      <c r="D15" s="5" t="s">
         <v>174</v>
       </c>
-      <c r="E15" s="7" t="n">
+      <c r="E15" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="F15" s="7" t="n">
+      <c r="F15" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="G15" s="4" t="n">
+      <c r="G15" s="5" t="n">
         <f aca="false">E15*2-F15</f>
         <v>0</v>
       </c>
-      <c r="H15" s="4"/>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4" t="n">
+      <c r="H15" s="5"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="5" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="5" t="s">
         <v>175</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="C16" s="5" t="s">
         <v>176</v>
       </c>
-      <c r="D16" s="4" t="s">
+      <c r="D16" s="5" t="s">
         <v>177</v>
       </c>
-      <c r="E16" s="7" t="n">
+      <c r="E16" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="F16" s="7" t="n">
+      <c r="F16" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G16" s="4" t="n">
+      <c r="G16" s="5" t="n">
         <f aca="false">E16*2-F16</f>
         <v>4</v>
       </c>
-      <c r="H16" s="4"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="8" t="s">
+      <c r="H16" s="5"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B18" s="9" t="s">
         <v>178</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:H16"/>
   <conditionalFormatting sqref="G2:G16">
-    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
+    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
       <formula>G2&gt;=8</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2459,75 +2475,75 @@
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="70"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="70"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="50"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="6" t="s">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="7" t="s">
         <v>126</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="7" t="s">
         <v>179</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="7" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="4" t="n">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="5" t="s">
         <v>181</v>
       </c>
-      <c r="C2" s="9"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4" t="n">
+      <c r="C2" s="10"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="5" t="s">
         <v>182</v>
       </c>
-      <c r="C3" s="9"/>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="n">
+      <c r="C3" s="10"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="5" t="s">
         <v>183</v>
       </c>
-      <c r="C4" s="9"/>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="n">
+      <c r="C4" s="10"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="5" t="s">
         <v>184</v>
       </c>
-      <c r="C5" s="9"/>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="n">
+      <c r="C5" s="10"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="5" t="s">
         <v>185</v>
       </c>
-      <c r="C6" s="9"/>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="n">
+      <c r="C6" s="10"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="5" t="s">
         <v>186</v>
       </c>
-      <c r="C7" s="9"/>
+      <c r="C7" s="10"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>